<commit_message>
Fees & Discounts TestRail import: drop 'Fees and Discounts V1 >' section prefix (use leaf section names)
</commit_message>
<xml_diff>
--- a/testrail-import/fees-discounts-v1-testrail-import.xlsx
+++ b/testrail-import/fees-discounts-v1-testrail-import.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Whole-WO Fee/Discount</t>
+          <t>Work Order — Whole-WO Fee/Discount</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Labor-line Fee/Discount</t>
+          <t>Work Order — Labor-line Fee/Discount</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order / Parts — Part-line Fee/Discount</t>
+          <t>Work Order / Parts — Part-line Fee/Discount</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Inline display (Lines tab)</t>
+          <t>Work Order — Inline display (Lines tab)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Inline display (Lines tab)</t>
+          <t>Work Order — Inline display (Lines tab)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Inline display (Lines tab)</t>
+          <t>Work Order — Inline display (Lines tab)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Inline display (Lines tab)</t>
+          <t>Work Order — Inline display (Lines tab)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Inline display (Lines tab)</t>
+          <t>Work Order — Inline display (Lines tab)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Statistics tab</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Statistics tab</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Statistics tab</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Statistics tab</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Statistics tab</t>
+          <t>Work Order — Statistics tab</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Financial Info card</t>
+          <t>Work Order — Financial Info card</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Financial Info card</t>
+          <t>Work Order — Financial Info card</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Financial Info card</t>
+          <t>Work Order — Financial Info card</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Sidebar 'Work Order Fee / Discount' card</t>
+          <t>Work Order — Sidebar 'Work Order Fee / Discount' card</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Sidebar 'Work Order Fee / Discount' card</t>
+          <t>Work Order — Sidebar 'Work Order Fee / Discount' card</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Parts page — breakdown modal</t>
+          <t>Parts page — breakdown modal</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Parts page — breakdown modal</t>
+          <t>Parts page — breakdown modal</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Parts page — breakdown modal</t>
+          <t>Parts page — breakdown modal</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Parts page — 'FEES &amp; DISCOUNTS' column</t>
+          <t>Parts page — 'FEES &amp; DISCOUNTS' column</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Edit an adjustment</t>
+          <t>Work Order — Edit an adjustment</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Edit an adjustment</t>
+          <t>Work Order — Edit an adjustment</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Edit an adjustment</t>
+          <t>Work Order — Edit an adjustment</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Remove an adjustment</t>
+          <t>Work Order — Remove an adjustment</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Remove an adjustment</t>
+          <t>Work Order — Remove an adjustment</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Remove an adjustment</t>
+          <t>Work Order — Remove an adjustment</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Multiple adjustments (stacking / netting)</t>
+          <t>Work Order — Multiple adjustments (stacking / netting)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Multiple adjustments (stacking / netting)</t>
+          <t>Work Order — Multiple adjustments (stacking / netting)</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Work Order — Multiple adjustments (stacking / netting)</t>
+          <t>Work Order — Multiple adjustments (stacking / netting)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab</t>
+          <t>Customer Fees &amp; Discounts tab</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer defaults → new work order</t>
+          <t>Customer defaults → new work order</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer defaults → new work order</t>
+          <t>Customer defaults → new work order</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4100,7 +4100,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer defaults lifecycle</t>
+          <t>Customer defaults lifecycle</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer defaults lifecycle</t>
+          <t>Customer defaults lifecycle</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer defaults lifecycle</t>
+          <t>Customer defaults lifecycle</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer defaults seeding</t>
+          <t>Customer defaults seeding</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab — permissions</t>
+          <t>Customer Fees &amp; Discounts tab — permissions</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer defaults — known bug</t>
+          <t>Customer defaults — known bug</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer Fees &amp; Discounts tab — negative</t>
+          <t>Customer Fees &amp; Discounts tab — negative</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — location</t>
+          <t>Template admin — location</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — list</t>
+          <t>Template admin — list</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -4535,7 +4535,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — create</t>
+          <t>Template admin — create</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — create</t>
+          <t>Template admin — create</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -4635,7 +4635,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — auto-apply</t>
+          <t>Template admin — auto-apply</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -4684,7 +4684,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — edit</t>
+          <t>Template admin — edit</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — delete</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — delete</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -4828,7 +4828,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — delete</t>
+          <t>Template admin — delete</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — scoping</t>
+          <t>Template admin — scoping</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — dialog fields</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — list</t>
+          <t>Template admin — list</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — validation</t>
+          <t>Template admin — validation</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — dialog fields</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — negative</t>
+          <t>Template admin — negative</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — permissions</t>
+          <t>Template admin — permissions</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Template admin — dialog fields</t>
+          <t>Template admin — dialog fields</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — template builder</t>
+          <t>Processing Fee — template builder</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — methods</t>
+          <t>Processing Fee — methods</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -5355,7 +5355,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — no Max Amount</t>
+          <t>Processing Fee — no Max Amount</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -5401,7 +5401,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — taxable + legal disclosure</t>
+          <t>Processing Fee — taxable + legal disclosure</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — no manual add</t>
+          <t>Processing Fee — no manual add</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — auto-apply</t>
+          <t>Processing Fee — auto-apply</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — customer default</t>
+          <t>Processing Fee — customer default</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — WO behavior</t>
+          <t>Processing Fee — WO behavior</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — calculation</t>
+          <t>Processing Fee — calculation</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — negative</t>
+          <t>Processing Fee — negative</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -5741,7 +5741,7 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — sign</t>
+          <t>Processing Fee — sign</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -5788,7 +5788,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — template edit independence</t>
+          <t>Processing Fee — template edit independence</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — calculation edge</t>
+          <t>Processing Fee — calculation edge</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Processing Fee — negative</t>
+          <t>Processing Fee — negative</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document (estimate/invoice)</t>
+          <t>Customer document (estimate/invoice)</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — per-line adjustments</t>
+          <t>Customer document — per-line adjustments</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — per-line adjustments</t>
+          <t>Customer document — per-line adjustments</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — amount format</t>
+          <t>Customer document — amount format</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — Adjustments block</t>
+          <t>Customer document — Adjustments block</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -6169,7 +6169,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — Adjustments block</t>
+          <t>Customer document — Adjustments block</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — Processing Fee phrase</t>
+          <t>Customer document — Processing Fee phrase</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — Shop Supplies (S14)</t>
+          <t>Customer document — Shop Supplies (S14)</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — Shop Supplies (S14)</t>
+          <t>Customer document — Shop Supplies (S14)</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — line-level $0 target</t>
+          <t>Customer document — line-level $0 target</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -6403,7 +6403,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Customer document — layout</t>
+          <t>Customer document — layout</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks sync</t>
+          <t>QuickBooks sync</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks sync</t>
+          <t>QuickBooks sync</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks sync — edge</t>
+          <t>QuickBooks sync — edge</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — mapping guard</t>
+          <t>QuickBooks — mapping guard</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — mapping guard</t>
+          <t>QuickBooks — mapping guard</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — mapping guard scope</t>
+          <t>QuickBooks — mapping guard scope</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — mapping guard (auto-apply)</t>
+          <t>QuickBooks — mapping guard (auto-apply)</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — mapping guard exceptions</t>
+          <t>QuickBooks — mapping guard exceptions</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — unmap recovery</t>
+          <t>QuickBooks — unmap recovery</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — Class</t>
+          <t>QuickBooks — Class</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — Class validation</t>
+          <t>QuickBooks — Class validation</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -6972,7 +6972,7 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — negative totals</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — negative totals</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — negative totals</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -7116,7 +7116,7 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks — negative totals</t>
+          <t>QuickBooks — negative totals</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; QuickBooks sync — tax</t>
+          <t>QuickBooks sync — tax</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log</t>
+          <t>History log</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
@@ -7259,7 +7259,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log</t>
+          <t>History log</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log</t>
+          <t>History log</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
@@ -7355,7 +7355,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log — visibility</t>
+          <t>History log — visibility</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log — visibility</t>
+          <t>History log — visibility</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -7454,7 +7454,7 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log — permission</t>
+          <t>History log — permission</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
@@ -7502,7 +7502,7 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log — Processing Fee</t>
+          <t>History log — Processing Fee</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -7551,7 +7551,7 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; History log — edit entry</t>
+          <t>History log — edit entry</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
@@ -7597,7 +7597,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
@@ -7759,7 +7759,7 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
@@ -7812,7 +7812,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
@@ -8077,7 +8077,7 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
@@ -8341,7 +8341,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -8397,7 +8397,7 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
@@ -8450,7 +8450,7 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Calculation contract</t>
+          <t>Calculation contract</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
@@ -8557,7 +8557,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
@@ -8609,7 +8609,7 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
@@ -8661,7 +8661,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
@@ -8713,7 +8713,7 @@
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
@@ -8817,7 +8817,7 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
@@ -8868,7 +8868,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
@@ -8975,7 +8975,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
@@ -9029,7 +9029,7 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Permissions (Story 13)</t>
+          <t>Permissions (Story 13)</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Feature-flag gating</t>
+          <t>Feature-flag gating</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Feature-flag gating</t>
+          <t>Feature-flag gating</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
@@ -9185,7 +9185,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Feature-flag gating</t>
+          <t>Feature-flag gating</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Validation / Edge</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Validation / Edge</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Validation / Edge</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
@@ -9395,7 +9395,7 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Validation / Edge</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Validation / Edge</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
@@ -9498,7 +9498,7 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Validation / Edge</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
@@ -9550,7 +9550,7 @@
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>Fees and Discounts V1 &gt; Validation / Edge</t>
+          <t>Validation / Edge</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Simple Flow + F&D: TestRail import files (VIU-word-free, no feature-flag preconditions) + permissions assessment
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/fees-discounts-v1-testrail-import.xlsx
+++ b/testrail-import/fees-discounts-v1-testrail-import.xlsx
@@ -512,9 +512,7 @@
         <is>
           <t>1. You are logged in as a role that has Work Orders: Create &amp; Edit and See Financial Data.
 2. An open (not Invoiced, not Paid) work order exists; you are viewing it and are NOT in history mode.
-3. You are on the work order's Lines tab.
-(Ref: FD-WO-001 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec: spec title = 'New Fee / Discount'; design mockup title = 'Add new fee/discount'. Authored to spec; flag the label difference at execution. Toolbar label 'Add Work Order Fee / Discount' is per S1-R1/S11-R4a comparison.</t>
+3. You are on the work order's Lines tab.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -563,9 +561,7 @@
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order with subtotal exactly $10,715.39 (or any known subtotal) is open on the Lines tab.
-(Ref: FD-WO-002 — VIU pending: verify on staging once deployed.)
-Note: Whole-WO Flat Amount base = the set amount, no quantity (open question #2 in requirements §14: no explicit Whole-WO Flat base row). Confirm button label per spec is 'Add Fee'; design mockup uses fixed 'Add' — flag.</t>
+2. An open work order with subtotal exactly $10,715.39 (or any known subtotal) is open on the Lines tab.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -620,9 +616,7 @@
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order with Work Order Total = $10,715.39 is open.
-(Ref: FD-WO-003 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec: the design preview always computes a percentage against the single flat WO Total and has NO base selector, whereas spec §5-R4 says whole-WO % must resolve against Net Labor / Net Parts / Subtotal depending on method. This is requirements open question #1. On staging, confirm which base is actually used; the −$857.23 number here matches the design's single-total math.</t>
+2. An open work order with Work Order Total = $10,715.39 is open.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -675,9 +669,7 @@
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order is open; the location's template library contains 'Fleet Standard Discount (−10%)'.
-(Ref: FD-WO-004 — VIU pending: verify on staging once deployed.)
-Note: Design mockup uses a 6-entry dropdown (Fleet Standard Discount, Loyalty Discount, Parts Handling Fee, Environmental Fee, Early Payment Discount, Labor Surcharge). Spec says the real product shares one location template library; substitute an actual staging template name if different. Taxable is not collected by the design's Add modal (design↔spec discrepancy #2).</t>
+2. An open work order is open; the location's template library contains 'Fleet Standard Discount (−10%)'.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -730,9 +722,7 @@
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order is open with the Add dialog freshly opened (all fields blank).
-(Ref: FD-WO-005 — VIU pending: verify on staging once deployed.)
-Note: The disabled-Add rule is the design's only validation gate; spec S2-N1/S2-N2 also expect inline error text on empty Name/Amount, which the design mockup does NOT render (design open item §10). Verify whether staging shows inline errors in addition to the disabled button.</t>
+2. An open work order is open with the Add dialog freshly opened (all fields blank).</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -787,9 +777,7 @@
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order whose relevant base for the fee is exactly $100.00 is open.
-(Ref: FD-WO-006 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec discrepancy #4: the design shows 'Max cap' unconditionally and even caps Flat Amount, while spec (S2-R24, §5-R6) shows Max Amount ONLY for a percentage method and never for Flat/Processing Fee. Field label is 'Max Amount (Optional)' per spec vs 'Max cap' in design. Also verify an entered Max Amount of 0 is treated as empty / no maximum (§5-R6, S2-R25).</t>
+2. An open work order whose relevant base for the fee is exactly $100.00 is open.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -839,9 +827,7 @@
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. The whole-WO Add dialog is open.
-(Ref: FD-WO-007 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec: the design mockup uses a fixed 'Add' button label that does NOT change with Type. Authored to spec S2-R27; flag the fixed label if staging matches the mockup.</t>
+2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -888,9 +874,7 @@
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. The whole-WO Add dialog is open.
-(Ref: FD-WO-008 — VIU pending: verify on staging once deployed.)
-Note: Verify whether staging surfaces an inline 'Name required' error (spec) or only keeps the button disabled (design).</t>
+2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -938,9 +922,7 @@
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. The whole-WO Add dialog is open with Name, Type='Fee', Calc type='Flat amount' set.
-(Ref: FD-WO-009 — VIU pending: verify on staging once deployed.)
-Note: Confirm minimum enforcement: Flat &lt; $0.01 and Percentage &lt; 0.01% are invalid (§5-R1).</t>
+2. The whole-WO Add dialog is open with Name, Type='Fee', Calc type='Flat amount' set.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -987,9 +969,7 @@
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. The whole-WO Add dialog is open.
-(Ref: FD-WO-010 — VIU pending: verify on staging once deployed.)
-Note: The design mockup does not model the &gt;100% discount validation (no inline error states). Verify the guard exists on staging.</t>
+2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1036,9 +1016,7 @@
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order with Net Labor total $200.00, Net Parts total $100.00, Shop Supplies $0.00 (so Subtotal = $300.00), no other adjustments.
-(Ref: FD-WO-011 — VIU pending: verify on staging once deployed.)
-Note: Design open question #1: the design Add modal only offers 'Percentage'/'Flat amount' with no base selector and computes % off a single flat total. Spec §5-R10 requires the four distinct whole-WO methods. Authored to spec; on staging confirm whether the base is a selectable Calculation type option or is chosen elsewhere.</t>
+2. An open work order with Net Labor total $200.00, Net Parts total $100.00, Shop Supplies $0.00 (so Subtotal = $300.00), no other adjustments.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1088,9 +1066,7 @@
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. A work order in Invoiced (or Paid) status is open.
-(Ref: FD-WO-012 — VIU pending: verify on staging once deployed.)
-Note: Also verify per-entry/per-row Edit/Delete 3-dot menus are hidden on Invoiced/Paid WOs (S3-N3).</t>
+2. A work order in Invoiced (or Paid) status is open.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1138,9 +1114,7 @@
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>1. Logged in as a role that HAS See Financial Data but does NOT have Work Orders: Create &amp; Edit.
-2. An open work order is open.
-(Ref: FD-WO-013 — VIU pending: verify on staging once deployed.)
-Note: Whole-WO add/edit/remove maps to Work Orders: Create &amp; Edit (S13-R3). Per requirements §10.4 the current build may use one WO-edit check rather than the split whole-WO vs line-level model — verify.</t>
+2. An open work order is open.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1186,9 +1160,7 @@
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. The whole-WO Add dialog is freshly open.
-(Ref: FD-WO-014 — VIU pending: verify on staging once deployed.)
-Note: Also verify the totals-load-failure preview text 'We couldn't load the figures to preview this selection.' (S2-R42) if a failure can be simulated.</t>
+2. The whole-WO Add dialog is freshly open.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1235,9 +1207,7 @@
       <c r="E16" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. The whole-WO Add dialog is open.
-(Ref: FD-WO-015 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec color conflict: the design mockup renders DISCOUNT amounts in green (--sv-success-text) and FEE amounts in amber/warning (--sv-warning-text), the OPPOSITE of spec S2-R33 (fee green, discount red). Authored the expected to spec; flag the mismatch and confirm the actual color on staging.</t>
+2. The whole-WO Add dialog is open.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1284,9 +1254,7 @@
       <c r="E17" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit and See Financial Data.
-2. An open work order with a labor line, e.g. Line 1 'Service - Perform LOF and inspection', is open on the Lines tab.
-(Ref: FD-LABOR-001 — VIU pending: verify on staging once deployed.)
-Note: Line-level add/edit/remove maps to Work Order Lines: Create &amp; Edit (S13-R4). Design mockup subtitle format is a scope link; spec exact string is 'Applying to: Line {N} Labor — {name}'.</t>
+2. An open work order with a labor line, e.g. Line 1 'Service - Perform LOF and inspection', is open on the Lines tab.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1335,9 +1303,7 @@
       <c r="E18" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a labor line whose gross labor price is exactly $150.00, no existing adjustments on that line.
-(Ref: FD-LABOR-002 — VIU pending: verify on staging once deployed.)
-Note: Default method for a labor line = % of Labor Total (S2-R22). Note the design Add modal lacks base-aware calc options (open question #1).</t>
+2. An open work order with a labor line whose gross labor price is exactly $150.00, no existing adjustments on that line.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1388,9 +1354,7 @@
       <c r="E19" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with two or more labor lines is open on the Lines tab.
-(Ref: FD-LABOR-003 — VIU pending: verify on staging once deployed.)
-Note: 'Add fee / discount' is NOT on the work-order line's right-click menu — it is the row 3-dot menu (S1 context note).</t>
+2. An open work order with two or more labor lines is open on the Lines tab.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1437,9 +1401,7 @@
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a labor line (any quantity/hours) is open.
-(Ref: FD-LABOR-004 — VIU pending: verify on staging once deployed.)
-Note: Contrast with Part Line Flat Amount, which IS per-item × quantity (see FD-PART-002).</t>
+2. An open work order with a labor line (any quantity/hours) is open.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1487,9 +1449,7 @@
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a labor line that carries a 10% fee adjustment resolving to a non-zero amount.
-(Ref: FD-LABOR-005 — VIU pending: verify on staging once deployed.)
-Note: Line-level adjustments show wherever their target shows, including a Needs Approval estimate (§5-R12).</t>
+2. An open work order with a labor line that carries a 10% fee adjustment resolving to a non-zero amount.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1538,9 +1498,7 @@
       <c r="E22" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a labor line that carries at least one fee/discount adjustment.
-(Ref: FD-LABOR-006 — VIU pending: verify on staging once deployed.)
-Note: Deleting a line/part removes its adjustments even though removal normally uses the Create &amp; Edit permission (this is a whole-record delete).</t>
+2. An open work order with a labor line that carries at least one fee/discount adjustment.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1588,9 +1546,7 @@
       <c r="E23" s="2" t="inlineStr">
         <is>
           <t>1. Logged in as a role with See Financial Data but WITHOUT Work Order Lines: Create &amp; Edit.
-2. An open work order with a labor line is open.
-(Ref: FD-LABOR-007 — VIU pending: verify on staging once deployed.)
-Note: Labor/part-line actions require Work Order Lines: Create &amp; Edit (S13-R4), distinct from the whole-WO permission (S13-R3).</t>
+2. An open work order with a labor line is open.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1637,9 +1593,7 @@
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a part, e.g. '(LF3620) Engine Oil Filter', is open on the Lines or Parts tab.
-(Ref: FD-PART-001 — VIU pending: verify on staging once deployed.)
-Note: Default method for a part = % of Parts Total (S2-R22). Design subtitle is a scope link; spec exact string is 'Applying to: Line {N} Part — ({part number}) {description}'.</t>
+2. An open work order with a part, e.g. '(LF3620) Engine Oil Filter', is open on the Lines or Parts tab.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1688,9 +1642,7 @@
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a part of quantity 3.
-(Ref: FD-PART-002 — VIU pending: verify on staging once deployed.)
-Note: Key edge behavior — Part Line Flat Amount is the only Flat Amount scope that multiplies by quantity. See FD-PART-008 for the qty=1 edge (−$5.00).</t>
+2. An open work order with a part of quantity 3.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1740,9 +1692,7 @@
       <c r="E26" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a requested (pending / not yet picked) part of quantity 2 at sell price $20.00 each.
-(Ref: FD-PART-003 — VIU pending: verify on staging once deployed.)
-Note: The part menu offers 'Add fee / discount' for both staged and requested parts (S1-R4). See FD-PART-005 for requested→received persistence.</t>
+2. An open work order with a requested (pending / not yet picked) part of quantity 2 at sell price $20.00 each.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1792,9 +1742,7 @@
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a part of quantity 3 at sell price $20.00 each (gross part total $60.00).
-(Ref: FD-PART-004 — VIU pending: verify on staging once deployed.)
-Note: Part Line percentage base uses the target's gross part total (before whole-WO nets).</t>
+2. An open work order with a part of quantity 3 at sell price $20.00 each (gross part total $60.00).</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1843,9 +1791,7 @@
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a requested part that already carries a % of Parts Total discount.
-(Ref: FD-PART-005 — VIU pending: verify on staging once deployed.)
-Note: Companion to FD-PART-003 (adding to a requested part).</t>
+2. An open work order with a requested part that already carries a % of Parts Total discount.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1893,9 +1839,7 @@
       <c r="E29" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a part carrying a discount that resolves to a non-zero amount.
-(Ref: FD-PART-006 — VIU pending: verify on staging once deployed.)
-Note: A part is billable when authorized, not declined, and still has quantity left (§5-R12).</t>
+2. An open work order with a part carrying a discount that resolves to a non-zero amount.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1944,9 +1888,7 @@
       <c r="E30" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a part that carries at least one adjustment.
-(Ref: FD-PART-007 — VIU pending: verify on staging once deployed.)
-Note: Same delete-cascade behavior as labor lines (FD-LABOR-006).</t>
+2. An open work order with a part that carries at least one adjustment.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1994,9 +1936,7 @@
       <c r="E31" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a part of quantity 1.
-(Ref: FD-PART-008 — VIU pending: verify on staging once deployed.)
-Note: Confirms quantity changes re-resolve a Part Line Flat Amount adjustment (§5-R14).</t>
+2. An open work order with a part of quantity 1.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2044,9 +1984,7 @@
       <c r="E32" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order where Line 1 labor carries a 'Line discount' of −5% resolving to −$26.08.
-(Ref: FD-INLINE-001 — VIU pending: verify on staging once deployed.)
-Note: Plain grey (not green/red) is correct outside the Add/Edit preview (S12-R1/R2).</t>
+2. An open work order where Line 1 labor carries a 'Line discount' of −5% resolving to −$26.08.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2094,9 +2032,7 @@
       <c r="E33" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order where part '(LF3620) Engine Oil Filter' carries a 'Parts Handling Fee' of +$3.75.
-(Ref: FD-INLINE-002 — VIU pending: verify on staging once deployed.)
-Note: Flat rate badge = signed dollar amount; percentage rate badge = signed percent with zeros removed (S3-R6/R7, S12-R4).</t>
+2. An open work order where part '(LF3620) Engine Oil Filter' carries a 'Parts Handling Fee' of +$3.75.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2144,9 +2080,7 @@
       <c r="E34" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order where the LF3620 part carries three adjustments: Part discount (−10%), Fleet discount (−5%), Parts Handling Fee (+$3.75).
-(Ref: FD-INLINE-003 — VIU pending: verify on staging once deployed.)
-Note: Same collapse/expand behavior applies to a labor line with 2+ adjustments.</t>
+2. An open work order where the LF3620 part carries three adjustments: Part discount (−10%), Fleet discount (−5%), Parts Handling Fee (+$3.75).</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2197,9 +2131,7 @@
       <c r="E35" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order where the LF3620 part has base total $58.47 plus adjustments −$6.49, −$2.92, +$3.75.
-(Ref: FD-INLINE-004 — VIU pending: verify on staging once deployed.)
-Note: Numbers taken from the design mockup (placeholder data); confirm actual stacked figures on staging.</t>
+2. An open work order where the LF3620 part has base total $58.47 plus adjustments −$6.49, −$2.92, +$3.75.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -2247,9 +2179,7 @@
       <c r="E36" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with at least one inline line-level adjustment.
-(Ref: FD-INLINE-005 — VIU pending: verify on staging once deployed.)
-Note: Design uses 'Edit/Delete' wording inline; spec says removal uses the Create &amp; Edit permission (not the Delete permission) despite the 'Delete' label (design↔spec wording note #7).</t>
+2. An open work order with at least one inline line-level adjustment.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2297,9 +2227,7 @@
       <c r="E37" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order with 5 adjustments across scopes is open.
-(Ref: FD-STATS-001 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec column-label difference: spec S4-R2 = '%' column; design mockup = 'Value' column. Authored to spec; flag the actual header on staging.</t>
+2. An open work order with 5 adjustments across scopes is open.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2348,9 +2276,7 @@
       <c r="E38" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order (e.g. S2-13274) with a whole-WO discount and line-level part/labor adjustments.
-(Ref: FD-STATS-002 — VIU pending: verify on staging once deployed.)
-Note: Scope hyperlink is a design affordance; confirm the exact jump/breakdown behavior on staging.</t>
+2. An open work order (e.g. S2-13274) with a whole-WO discount and line-level part/labor adjustments.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2399,9 +2325,7 @@
       <c r="E39" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order with adjustments: Work order discount −$857.23, Part discount −$649.00, Fleet discount −$292.00, Parts Handling Fee +$3.75, Line discount −$260.77.
-(Ref: FD-STATS-003 — VIU pending: verify on staging once deployed.)
-Note: The design mockup's Stats total placeholder (−$1,198.02) disagrees with its Financial Info total (−$2,055.25) for the same '(5)' set — treat as mock placeholder inconsistency (design §3 warning). Expected here uses the correct signed sum −$2,055.25.</t>
+2. An open work order with adjustments: Work order discount −$857.23, Part discount −$649.00, Fleet discount −$292.00, Parts Handling Fee +$3.75, Line discount −$260.77.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2449,9 +2373,7 @@
       <c r="E40" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order to which you add three adjustments in a known order: (a) Adjustment A first, (b) Adjustment B second, (c) Adjustment C third.
-(Ref: FD-STATS-004 — VIU pending: verify on staging once deployed.)
-Note: The Group-A task brief mentions 'descending build order', but spec §5-R9 is explicit that WO screens (sidebar card, Financial Info, line table, Statistics tab) list adjustments in creation order OLDEST first. Authored to spec — flag the wording difference and confirm the actual order on staging.</t>
+2. An open work order to which you add three adjustments in a known order: (a) Adjustment A first, (b) Adjustment B second, (c) Adjustment C third.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2498,9 +2420,7 @@
       <c r="E41" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order with zero fee/discount adjustments of any scope.
-(Ref: FD-STATS-005 — VIU pending: verify on staging once deployed.)
-Note: Mirrors the Financial Info row hidden state (S3-N2) and the sidebar card hidden state (S3-N1).</t>
+2. An open work order with zero fee/discount adjustments of any scope.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2546,9 +2466,7 @@
       <c r="E42" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order with 5 adjustments (any scopes) netting to −$2,055.25.
-(Ref: FD-FIN-001 — VIU pending: verify on staging once deployed.)
-Note: This is a distinct count/total from the sidebar 'Work Order Fee / Discount' card, which lists whole-WO adjustments only.</t>
+2. An open work order with 5 adjustments (any scopes) netting to −$2,055.25.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2597,9 +2515,7 @@
       <c r="E43" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order with 5 adjustments as in FD-FIN-001.
-(Ref: FD-FIN-002 — VIU pending: verify on staging once deployed.)
-Note: Financial Info card is read-only for adjustments (key decision, §3 of spec). Scope disambiguation uses a suffix e.g. '(LF3620)'.</t>
+2. An open work order with 5 adjustments as in FD-FIN-001.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2647,9 +2563,7 @@
       <c r="E44" s="2" t="inlineStr">
         <is>
           <t>1. Variant (a): logged in with See Financial Data, an open WO with zero adjustments.
-2. Variant (b): logged in as a role WITHOUT See Financial Data, an open WO with adjustments.
-(Ref: FD-FIN-003 — VIU pending: verify on staging once deployed.)
-Note: See Financial Data gates visibility of all fee/discount dollar amounts across surfaces (S13-R2/N1).</t>
+2. Variant (b): logged in as a role WITHOUT See Financial Data, an open WO with adjustments.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2696,9 +2610,7 @@
       <c r="E45" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data and Work Orders: Create &amp; Edit.
-2. An open work order with a whole-WO 'Early Payment Discount' of −8% resolving to −$857.23, plus some line-level adjustments.
-(Ref: FD-FIN-004 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec color note: the design renders the discount amount in green (--sv-success-text); spec S12-R1 says sidebar amounts are plain grey. Authored to spec (plain grey); flag the color. Card title is 'Work Order Fee / Discount' in the final mockup vs 'WO Fees &amp; Discounts' in v1 mockup / spec S3-R3.</t>
+2. An open work order with a whole-WO 'Early Payment Discount' of −8% resolving to −$857.23, plus some line-level adjustments.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2748,9 +2660,7 @@
         <is>
           <t>1. Logged in with See Financial Data + Work Orders: Create &amp; Edit.
 2. Variant (a): an open WO with only line-level adjustments and NO whole-WO adjustments.
-3. Variant (b): an open WO with at least one whole-WO adjustment.
-(Ref: FD-FIN-005 — VIU pending: verify on staging once deployed.)
-Note: Design↔spec: the v1 mockup card includes an 'Add Fee / Discount' secondary button, which contradicts spec S3-R10 (no Add control on the card). Authored to spec (no Add control); flag if staging shows an in-card Add button.</t>
+3. Variant (b): an open WO with at least one whole-WO adjustment.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2797,9 +2707,7 @@
       <c r="E47" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. A Parts page / WO parts view is open with part '#37346 Mobil 1 5W20' carrying exactly one adjustment 'Military Discount' −10%.
-(Ref: FD-PCOL-001 — VIU pending: verify on staging once deployed.)
-Note: The 'Fees &amp; Discounts' column shows only on a part sale / parts view when the flag is on (S11-R7). Core-charge rows have an empty column (S11-R8).</t>
+2. A Parts page / WO parts view is open with part '#37346 Mobil 1 5W20' carrying exactly one adjustment 'Military Discount' −10%.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2846,9 +2754,7 @@
       <c r="E48" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. Parts page open with part '#55073 Mobil 1 5W20' carrying three adjustments (first = 'Parts Handling Fee' 2%).
-(Ref: FD-PCOL-002 — VIU pending: verify on staging once deployed.)
-Note: Badge count N is the number of adjustments AFTER the first (so 3 total → '+2').</t>
+2. Parts page open with part '#55073 Mobil 1 5W20' carrying three adjustments (first = 'Parts Handling Fee' 2%).</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2895,9 +2801,7 @@
       <c r="E49" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data and the relevant change permission.
-2. Parts page open with part '#28439 Fleetguard FF5421' carrying no adjustments, on an editable sale/WO.
-(Ref: FD-PCOL-003 — VIU pending: verify on staging once deployed.)
-Note: The '+ Add' button is disabled when the sale/WO cannot be edited (see FD-PCOL-008).</t>
+2. Parts page open with part '#28439 Fleetguard FF5421' carrying no adjustments, on an editable sale/WO.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2945,9 +2849,7 @@
       <c r="E50" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. Parts page open with part '#55073 Mobil 1 5W20' carrying three adjustments (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).
-(Ref: FD-PCOL-004 — VIU pending: verify on staging once deployed.)
-Note: The WO-line/customer variant of this breakdown omits the Max Amount column and the per-row trash (read-only); the Parts-page variant adds both (design §8).</t>
+2. Parts page open with part '#55073 Mobil 1 5W20' carrying three adjustments (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2997,9 +2899,7 @@
       <c r="E51" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. The #55073 breakdown modal from FD-PCOL-004 is open (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).
-(Ref: FD-PCOL-005 — VIU pending: verify on staging once deployed.)
-Note: For a single-adjustment part (#37346 Military Discount −$6.53) the Net adjustment equals that one amount (−$6.53).</t>
+2. The #55073 breakdown modal from FD-PCOL-004 is open (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3044,9 +2944,7 @@
       <c r="E52" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with the relevant change permission + See Financial Data.
-2. Parts page open with part #37346 carrying exactly ONE adjustment; the editable breakdown modal is open.
-(Ref: FD-PCOL-006 — VIU pending: verify on staging once deployed.)
-Note: Removal uses the Create &amp; Edit permission, NOT the Delete permission (S13-R7). Per-row remove is shown only when the sale/WO can be edited (S11-R14).</t>
+2. Parts page open with part #37346 carrying exactly ONE adjustment; the editable breakdown modal is open.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3095,9 +2993,7 @@
       <c r="E53" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. Parts page open for an Invoiced/Paid (non-editable) sale/WO with a part that has no adjustments.
-(Ref: FD-PCOL-007 — VIU pending: verify on staging once deployed.)
-Note: Ties to the Invoiced/Paid lifecycle gate (S1-N1, S3-R1b).</t>
+2. Parts page open for an Invoiced/Paid (non-editable) sale/WO with a part that has no adjustments.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3144,9 +3040,7 @@
       <c r="E54" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with the relevant change permission + See Financial Data.
-2. An open work order with an existing whole-WO percentage discount adjustment.
-(Ref: FD-EDIT-001 — VIU pending: verify on staging once deployed.)
-Note: Design open item #10: the mockups contain NO Edit-dialog markup and do not show which fields are locked. Authored strictly to spec S2-R4/R5/R8; verify locked-field behavior on staging. Confirm button label on edit = 'Save' (S2-R28).</t>
+2. An open work order with an existing whole-WO percentage discount adjustment.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3197,9 +3091,7 @@
       <c r="E55" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with the relevant change permission + See Financial Data.
-2. An open work order with an existing percentage adjustment whose base total has since changed (e.g. a line was added).
-(Ref: FD-EDIT-002 — VIU pending: verify on staging once deployed.)
-Note: Verify re-resolution uses current (not original) totals.</t>
+2. An open work order with an existing percentage adjustment whose base total has since changed (e.g. a line was added).</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -3250,9 +3142,7 @@
       <c r="E56" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with the relevant change permission + See Financial Data.
-2. An open work order with an existing adjustment; a condition that forces a save failure can be simulated (e.g. server error).
-(Ref: FD-EDIT-003 — VIU pending: verify on staging once deployed.)
-Note: The design mockups model no error/toast states; this is spec-driven (S2-R30, §7 toast table).</t>
+2. An open work order with an existing adjustment; a condition that forces a save failure can be simulated (e.g. server error).</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3300,9 +3190,7 @@
       <c r="E57" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order with a whole-WO discount named 'Early Payment Discount'.
-(Ref: FD-REMOVE-001 — VIU pending: verify on staging once deployed.)
-Note: Design uses the label 'Delete' on the sidebar/inline ⋯ menus but the spec confirm dialog is titled 'Remove Fee / Discount' with a 'Remove' button; the design mockups do NOT model the confirm dialog (§10). Authored to spec — flag the label mismatch and confirm the dialog exists on staging.</t>
+2. An open work order with a whole-WO discount named 'Early Payment Discount'.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3352,9 +3240,7 @@
       <c r="E58" s="2" t="inlineStr">
         <is>
           <t>1. Logged in as a role that HAS Work Orders: Create &amp; Edit and See Financial Data but does NOT have the separate 'Delete' permission.
-2. An open work order with a whole-WO adjustment.
-(Ref: FD-REMOVE-002 — VIU pending: verify on staging once deployed.)
-Note: Key permission nuance: 'Delete' permission is for whole records (WO, labor line, part); removing an adjustment is part of 'Create and Edit' (S13-R7). For a line/part adjustment the required permission is Work Order Lines: Create &amp; Edit (S13-R4).</t>
+2. An open work order with a whole-WO adjustment.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3403,9 +3289,7 @@
       <c r="E59" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order where a part carries a 'Fleet discount' adjustment shown inline.
-(Ref: FD-REMOVE-003 — VIU pending: verify on staging once deployed.)
-Note: If removing brings the count down to one adjustment, the 'Show N more' toggle should disappear.</t>
+2. An open work order where a part carries a 'Fleet discount' adjustment shown inline.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -3455,9 +3339,7 @@
       <c r="E60" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Order Lines: Create &amp; Edit + See Financial Data.
-2. An open work order with a part of gross part total exactly $100.00.
-(Ref: FD-STACK-001 — VIU pending: verify on staging once deployed.)
-Note: Critical calc rule: line-level percentages all resolve against the same gross base — they never compound on each other (§5-R5).</t>
+2. An open work order with a part of gross part total exactly $100.00.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3510,9 +3392,7 @@
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit, Work Order Lines: Create &amp; Edit, and See Financial Data.
 2. An open work order with Gross Labor $200.00 and Gross Parts $100.00, no shop supplies.
-3. A Labor Line 10% discount already applied (Step 1: −$20.00, so Net Labor = $180.00).
-(Ref: FD-STACK-002 — VIU pending: verify on staging once deployed.)
-Note: Uses the spec's own §5 worked example. Confirms three-step resolve order and no compounding between whole-WO adjustments.</t>
+3. A Labor Line 10% discount already applied (Step 1: −$20.00, so Net Labor = $180.00).</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3562,9 +3442,7 @@
       <c r="E62" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with Work Orders: Create &amp; Edit + See Financial Data.
-2. An open work order; the location library has a 'Parts Handling Fee' template.
-(Ref: FD-STACK-003 — VIU pending: verify on staging once deployed.)
-Note: This is intentional manual re-application, distinct from the auto-apply + customer-default DOUBLE-ADD bug (requirements open question #4), which is a known defect, not a spec requirement.</t>
+2. An open work order; the location library has a 'Parts Handling Fee' template.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3612,9 +3490,7 @@
       <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. A test customer named ZZAUTOTEST Customer exists with exactly 2 default fees/discounts linked.
-2. You are logged in with Customer Management: Create &amp; Edit and Manage AP/AR permissions.
-(Ref: FD-CUST-001 — VIU pending: verify on staging once deployed.)
-Note: Count in parentheses = number of default links on the customer, not adjustments on work orders.</t>
+2. You are logged in with Customer Management: Create &amp; Edit and Manage AP/AR permissions.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3662,9 +3538,7 @@
       <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. A customer with at least 1 default fee/discount exists.
-2. You have Customer Management: Create &amp; Edit + Manage AP/AR.
-(Ref: FD-CUST-002 — VIU pending: verify on staging once deployed.)
-Note: Customer card uses "Add Fee/Discount" (no spaces); WO/template dialogs use "Add Fee / Discount" (with spaces) — keep both exact (S9-R... exact-text note).</t>
+2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3714,9 +3588,7 @@
       <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. A location template named "ZZAUTOTEST Fleet Discount" (Discount, % of Subtotal, 10%) exists and is NOT yet linked to the test customer.
-2. You have Customer Management: Create &amp; Edit + Manage AP/AR.
-(Ref: FD-CUST-003 — VIU pending: verify on staging once deployed.)
-Note: Toast for one default is the generic "Fee / discount added." — it does NOT vary by type (§7 toast table).</t>
+2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3766,9 +3638,7 @@
       <c r="E66" s="2" t="inlineStr">
         <is>
           <t>1. At least 3 templates exist that are NOT yet linked to the test customer.
-2. You have Customer Management: Create &amp; Edit + Manage AP/AR.
-(Ref: FD-CUST-004 — VIU pending: verify on staging once deployed.)
-Note: Plural toast pattern is "[N] fees / discounts added." per §7 toast table.</t>
+2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3817,9 +3687,7 @@
       <c r="E67" s="2" t="inlineStr">
         <is>
           <t>1. The location has: (a) a template already linked to this customer, (b) an unlinked Fee/Discount template, and (c) an unlinked Processing Fee template.
-2. You have Customer Management: Create &amp; Edit + Manage AP/AR.
-(Ref: FD-CUST-005 — VIU pending: verify on staging once deployed.)
-Note: This differs from the WO template picker, which NEVER lists a Processing Fee (S8-N2). Flag if staging shows raw "processing_fee" instead of "Fee".</t>
+2. You have Customer Management: Create &amp; Edit + Manage AP/AR.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3866,8 +3734,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>1. Every location template is already linked to the test customer (or the location has no templates).
-(Ref: FD-CUST-006 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. Every location template is already linked to the test customer (or the location has no templates).</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3912,9 +3779,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>1. The customer has at least 1 default fee/discount.
-(Ref: FD-CUST-007 — VIU pending: verify on staging once deployed.)
-Note: Removing a customer default is intentionally no-confirm (S9-R24), unlike deleting a template (S7-R20 has a confirm).</t>
+          <t>1. The customer has at least 1 default fee/discount.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3963,8 +3828,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>1. The customer has zero default fees/discounts.
-(Ref: FD-CUST-008 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. The customer has zero default fees/discounts.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4010,9 +3874,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>1. The customer has a default "ZZAUTOTEST Fleet Discount" (Discount, % of Subtotal, 10%, non-taxable).
-(Ref: FD-CUST-009 — VIU pending: verify on staging once deployed.)
-Note: The adjustment is an independent copy; the WO surfaces are covered by Group A — this case focuses on the customer-default → WO seeding and independence.</t>
+          <t>1. The customer has a default "ZZAUTOTEST Fleet Discount" (Discount, % of Subtotal, 10%, non-taxable).</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -4060,9 +3922,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>1. The customer has a default "ZZAUTOTEST 10% Fee" (Fee, % of Subtotal, 10%, taxable).
-(Ref: FD-CUST-010 — VIU pending: verify on staging once deployed.)
-Note: Uses spec calc rule §5-R3.</t>
+          <t>1. The customer has a default "ZZAUTOTEST 10% Fee" (Fee, % of Subtotal, 10%, taxable).</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4110,8 +3970,7 @@
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>1. The customer has a default "ZZAUTOTEST Fleet Discount".
-2. An OPEN work order for that customer already carries the auto-added adjustment from this default.
-(Ref: FD-CUST-011 — VIU pending: verify on staging once deployed.)</t>
+2. An OPEN work order for that customer already carries the auto-added adjustment from this default.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -4158,9 +4017,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>1. A template "ZZAUTOTEST Fleet Discount" is a default on the customer AND has been auto-added to an existing OPEN work order.
-(Ref: FD-CUST-012 — VIU pending: verify on staging once deployed.)
-Note: Deleting the template drops template + default links but NOT existing WO adjustments — matches the task's stated rule.</t>
+          <t>1. A template "ZZAUTOTEST Fleet Discount" is a default on the customer AND has been auto-added to an existing OPEN work order.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4208,8 +4065,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>1. A disposable ZZAUTOTEST customer has at least 1 default fee/discount linked.
-(Ref: FD-CUST-013 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A disposable ZZAUTOTEST customer has at least 1 default fee/discount linked.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -4255,8 +4111,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>1. The location has exactly 2 templates marked auto-apply and 1 template not auto-apply.
-(Ref: FD-CUST-014 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. The location has exactly 2 templates marked auto-apply and 1 template not auto-apply.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4302,9 +4157,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>1. A ZZAUTOTEST role is assigned to Tech (exact-user-match) with Customer Management: Create &amp; Edit ON but Manage Accounts Payable and Receivable OFF.
-(Ref: FD-CUST-015 — VIU pending: verify on staging once deployed.)
-Note: CAUTION: Story 13 Custom-Roles model (SV-7388) may not be live on staging yet — record what staging actually enforces and flag divergence. Restore Tech to Time Clock (role 77b069d1-...) after.</t>
+          <t>1. A ZZAUTOTEST role is assigned to Tech (exact-user-match) with Customer Management: Create &amp; Edit ON but Manage Accounts Payable and Receivable OFF.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -4322,7 +4175,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>S13-R9, S13-N3 SV-7388</t>
+          <t>S13-R9, S13-N3</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
@@ -4351,9 +4204,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>1. A template "ZZAUTOTEST Env Fee" is marked auto-apply at the location AND is a default on the test customer.
-(Ref: FD-CUST-016 — VIU pending: verify on staging once deployed.)
-Note: A double-add is a KNOWN DEFECT tracked separately, not a spec requirement. Report actual behavior.</t>
+          <t>1. A template "ZZAUTOTEST Env Fee" is marked auto-apply at the location AND is a default on the test customer.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -4399,9 +4250,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>1. A way to force a server error (e.g., simulate a network/API failure) on the add or remove call.
-(Ref: FD-CUST-017 — VIU pending: verify on staging once deployed.)
-Note: Unlike WO/template save failures, customer-default failures use the generic system error, not a custom message.</t>
+          <t>1. A way to force a server error (e.g., simulate a network/API failure) on the add or remove call.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -4447,9 +4296,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>1. You have Settings → Finance access.
-(Ref: FD-TMPL-001 — VIU pending: verify on staging once deployed.)
-Note: The admin Fees &amp; Discounts page is NOT in the HTML mockups — confirm its exact placement live.</t>
+          <t>1. You have Settings → Finance access.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4495,8 +4342,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>1. The location has at least 1 template.
-(Ref: FD-TMPL-002 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. The location has at least 1 template.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -4543,9 +4389,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>1. You are on Administration → Service → Fees &amp; Discounts.
-(Ref: FD-TMPL-003 — VIU pending: verify on staging once deployed.)
-Note: Create confirm button label is FIXED "Add Fee / Discount" for any type (S7-R17), unlike the WO dialog which flips to "Add Fee"/"Add Discount" (S2-R27).</t>
+          <t>1. You are on Administration → Service → Fees &amp; Discounts.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4595,8 +4439,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin Fees &amp; Discounts page.
-(Ref: FD-TMPL-004 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. On the admin Fees &amp; Discounts page.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -4643,8 +4486,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>1. You can create a template and then a new work order at the same location.
-(Ref: FD-TMPL-005 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. You can create a template and then a new work order at the same location.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4692,8 +4534,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>1. A Fee template "ZZAUTOTEST Shop Fee" exists.
-(Ref: FD-TMPL-006 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A Fee template "ZZAUTOTEST Shop Fee" exists.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -4741,9 +4582,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>1. A template that is NOT a default for any customer exists.
-(Ref: FD-TMPL-007 — VIU pending: verify on staging once deployed.)
-Note: The remove-confirm dialog is not in the HTML mockups; verify exact copy live.</t>
+          <t>1. A template that is NOT a default for any customer exists.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -4790,8 +4629,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>1. A template is set as a default for exactly 2 customers.
-(Ref: FD-TMPL-008 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A template is set as a default for exactly 2 customers.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -4836,8 +4674,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>1. A template has been applied to an OPEN work order as an adjustment.
-(Ref: FD-TMPL-009 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A template has been applied to an OPEN work order as an adjustment.</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -4884,9 +4721,7 @@
       <c r="E89" s="2" t="inlineStr">
         <is>
           <t>1. The location has: a "% of Labor Total" template, a "% of Parts Total" template, and a Flat Amount template.
-2. A work order with at least one labor line and one part exists.
-(Ref: FD-TMPL-010 — VIU pending: verify on staging once deployed.)
-Note: Matches the task's scoping rule (labour templates only accepted by labour modals, not parts, and vice versa). Loom transcript confirms scope filtering.</t>
+2. A work order with at least one labor line and one part exists.</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -4936,9 +4771,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin Fees &amp; Discounts create dialog.
-(Ref: FD-TMPL-011 — VIU pending: verify on staging once deployed.)
-Note: Design mockups show a "Max cap" always rendered (design-notes §10 item 4) — flag if staging shows Max Amount for Flat too.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -4986,8 +4819,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>1. The location has zero templates.
-(Ref: FD-TMPL-012 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. The location has zero templates.</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -5032,8 +4864,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin Fees &amp; Discounts create dialog.
-(Ref: FD-TMPL-013 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -5079,9 +4910,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin Fees &amp; Discounts create dialog with Type = Fee or Discount.
-(Ref: FD-TMPL-014 — VIU pending: verify on staging once deployed.)
-Note: Processing Fee has different method options (Flat Amount, % of Grand Total) — see FD-PROC-002.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog with Type = Fee or Discount.</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -5127,8 +4956,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>1. A way to force a save failure on the template create/edit call.
-(Ref: FD-TMPL-015 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A way to force a save failure on the template create/edit call.</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -5173,9 +5001,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>1. A ZZAUTOTEST role is assigned to Tech (exact-user-match) WITHOUT Settings → Finance.
-(Ref: FD-TMPL-016 — VIU pending: verify on staging once deployed.)
-Note: CURRENT-BUILD DIFFERENCE (§10.4/S7-R7b): today the page may show to any user with a location; S13-R8 tightens it to Settings → Finance. Record actual gating. Restore Tech to Time Clock after.</t>
+          <t>1. A ZZAUTOTEST role is assigned to Tech (exact-user-match) WITHOUT Settings → Finance.</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -5220,8 +5046,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin Fees &amp; Discounts create dialog.
-(Ref: FD-TMPL-017 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -5267,9 +5092,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin Fees &amp; Discounts create dialog.
-(Ref: FD-PROC-001 — VIU pending: verify on staging once deployed.)
-Note: Processing Fee UI is absent from the HTML mockups — verify live.</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog.</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -5314,8 +5137,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin Fees &amp; Discounts create dialog with Type = "Processing Fee".
-(Ref: FD-PROC-002 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. On the admin Fees &amp; Discounts create dialog with Type = "Processing Fee".</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -5362,8 +5184,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin create dialog with Type = Processing Fee.
-(Ref: FD-PROC-003 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. On the admin create dialog with Type = Processing Fee.</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -5408,9 +5229,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>1. On the admin create dialog with Type = Processing Fee.
-(Ref: FD-PROC-004 — VIU pending: verify on staging once deployed.)
-Note: OPEN QUESTION (§14 item 5): the disclosure's literal text is NOT in the exported spec — capture the exact wording from the live dialog before asserting it. Spec copy says "toggle" but the control is the Yes/No dropdown.</t>
+          <t>1. On the admin create dialog with Type = Processing Fee.</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -5459,9 +5278,7 @@
       <c r="E101" s="2" t="inlineStr">
         <is>
           <t>1. A Processing Fee template exists.
-2. An open work order is available.
-(Ref: FD-PROC-005 — VIU pending: verify on staging once deployed.)
-Note: Processing Fee reaches a WO only via auto-apply (S8-R14) or a customer default (S8-R15).</t>
+2. An open work order is available.</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -5507,8 +5324,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>1. A Processing Fee template "ZZAUTOTEST Proc Fee" (Flat Amount $5.00, taxable Yes) is marked auto-apply.
-(Ref: FD-PROC-006 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A Processing Fee template "ZZAUTOTEST Proc Fee" (Flat Amount $5.00, taxable Yes) is marked auto-apply.</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -5554,8 +5370,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>1. A Processing Fee template is set as a default on the test customer.
-(Ref: FD-PROC-007 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A Processing Fee template is set as a default on the test customer.</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -5601,9 +5416,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>1. An open WO carries a Processing Fee (via auto-apply or customer default).
-(Ref: FD-PROC-008 — VIU pending: verify on staging once deployed.)
-Note: CURRENT-BUILD DIFFERENCE (§14 item 6): the current build may still show an Edit control that fails (S8-R17). Record actual behavior.</t>
+          <t>1. An open WO carries a Processing Fee (via auto-apply or customer default).</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -5651,9 +5464,7 @@
       <c r="E105" s="2" t="inlineStr">
         <is>
           <t>1. A Processing Fee template "ZZAUTOTEST 3% Proc" (% of Grand Total, 3%, taxable Yes) auto-applies.
-2. A work order exists whose net subtotal (after line-level adjustments) = $300.00 and pre-fee tax = $24.00 (so Grand Total base = $324.00).
-(Ref: FD-PROC-009 — VIU pending: verify on staging once deployed.)
-Note: Uses the spec's worked example directly.</t>
+2. A work order exists whose net subtotal (after line-level adjustments) = $300.00 and pre-fee tax = $24.00 (so Grand Total base = $324.00).</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -5700,9 +5511,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>1. Ability to submit template data (via UI edge case or API) for a Processing Fee carrying a Max Amount, or a method other than Flat Amount / % of Grand Total.
-(Ref: FD-PROC-010 — VIU pending: verify on staging once deployed.)
-Note: The UI hides these options; this guards data sent from outside the product.</t>
+          <t>1. Ability to submit template data (via UI edge case or API) for a Processing Fee carrying a Max Amount, or a method other than Flat Amount / % of Grand Total.</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -5748,8 +5557,7 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>1. A Processing Fee template exists and is on a WO.
-(Ref: FD-PROC-011 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A Processing Fee template exists and is on a WO.</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -5795,8 +5603,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>1. A Processing Fee template auto-applied to an existing OPEN work order (e.g. Flat $5.00).
-(Ref: FD-PROC-012 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A Processing Fee template auto-applied to an existing OPEN work order (e.g. Flat $5.00).</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -5843,8 +5650,7 @@
       <c r="E109" s="2" t="inlineStr">
         <is>
           <t>1. Two Processing Fee templates (both % of Grand Total) auto-apply to one work order.
-2. Net subtotal $300.00, pre-fee tax $24.00 → Grand Total base $324.00.
-(Ref: FD-PROC-013 — VIU pending: verify on staging once deployed.)</t>
+2. Net subtotal $300.00, pre-fee tax $24.00 → Grand Total base $324.00.</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -5890,9 +5696,7 @@
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>1. Ability to submit a Processing Fee with a non-empty minimum amount (no UI control exists; guard for external data).
-(Ref: FD-PROC-014 — VIU pending: verify on staging once deployed.)
-Note: Min Amount exists only in the data model; both dialogs always send it empty (null).</t>
+          <t>1. Ability to submit a Processing Fee with a non-empty minimum amount (no UI control exists; guard for external data).</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -5936,9 +5740,7 @@
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>1. A work order has whole-WO and line-level adjustments and can produce both an estimate and an invoice.
-(Ref: FD-DOC-001 — VIU pending: verify on staging once deployed.)
-Note: No customer estimate/invoice view exists in the HTML mockups — verify layout live.</t>
+          <t>1. A work order has whole-WO and line-level adjustments and can produce both an estimate and an invoice.</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -5984,8 +5786,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>1. A WO has a labor line with a "Shop Supply Fee" (% of Labor Total, fee) and a labor-line discount.
-(Ref: FD-DOC-002 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO has a labor line with a "Shop Supply Fee" (% of Labor Total, fee) and a labor-line discount.</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -6032,8 +5833,7 @@
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>1. A WO part has a percentage part-line adjustment and another part has a Flat Amount part-line adjustment.
-(Ref: FD-DOC-003 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO part has a percentage part-line adjustment and another part has a Flat Amount part-line adjustment.</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -6079,9 +5879,7 @@
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>1. A WO has both a fee and a discount adjustment.
-(Ref: FD-DOC-004 — VIU pending: verify on staging once deployed.)
-Note: Note this differs from WO screens, which use a signed minus (e.g. "−$26.08") in plain grey.</t>
+          <t>1. A WO has both a fee and a discount adjustment.</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -6128,8 +5926,7 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>1. A WO has 3 whole-WO adjustments created in a known order, including a % of Subtotal and a Flat Amount.
-(Ref: FD-DOC-005 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO has 3 whole-WO adjustments created in a known order, including a % of Subtotal and a Flat Amount.</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -6176,9 +5973,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>1. A WO has three separate "Shop Supply Fee" line-level fees (same name+type) across different lines.
-(Ref: FD-DOC-006 — VIU pending: verify on staging once deployed.)
-Note: Grouping is ONLY on the customer document; WO line table lists each one by one (Story 3).</t>
+          <t>1. A WO has three separate "Shop Supply Fee" line-level fees (same name+type) across different lines.</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -6224,8 +6019,7 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>1. A WO carries a % of Grand Total Processing Fee.
-(Ref: FD-DOC-007 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO carries a % of Grand Total Processing Fee.</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -6269,8 +6063,7 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>1. A WO whose total shop supplies = $0.00.
-(Ref: FD-DOC-008 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO whose total shop supplies = $0.00.</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -6317,8 +6110,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>1. A WO that currently has $0.00 shop supplies (Shop Supplies hidden on customer views).
-(Ref: FD-DOC-009 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO that currently has $0.00 shop supplies (Shop Supplies hidden on customer views).</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -6363,8 +6155,7 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>1. A WO labor line with an adjustment is set to declined/not-billable.
-(Ref: FD-DOC-010 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO labor line with an adjustment is set to declined/not-billable.</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -6410,8 +6201,7 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>1. A WO with labor, parts, shop supplies (&gt; $0.00), and whole-WO adjustments.
-(Ref: FD-DOC-011 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO with labor, parts, shop supplies (&gt; $0.00), and whole-WO adjustments.</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -6456,9 +6246,7 @@
       <c r="E122" s="2" t="inlineStr">
         <is>
           <t>1. Location has an active QuickBooks connection with mapped Fee and Discount items.
-2. A WO with one fee (+$10.00) and one discount (−$20.00) is invoiced.
-(Ref: FD-QB-001 — VIU pending: verify on staging once deployed.)
-Note: QuickBooks sync is backend; verify via the QuickBooks side or the sync payload.</t>
+2. A WO with one fee (+$10.00) and one discount (−$20.00) is invoiced.</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -6506,8 +6294,7 @@
       <c r="E123" s="2" t="inlineStr">
         <is>
           <t>1. QuickBooks connected with a mapped Fee item and Discount item.
-2. A WO has a fee named "Hazmat Disposal Fee"; the WO is invoiced.
-(Ref: FD-QB-002 — VIU pending: verify on staging once deployed.)</t>
+2. A WO has a fee named "Hazmat Disposal Fee"; the WO is invoiced.</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -6553,8 +6340,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; a WO has an adjustment that resolves to $0.00 (e.g. target not billable, or $0 base).
-(Ref: FD-QB-003 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. QuickBooks connected; a WO has an adjustment that resolves to $0.00 (e.g. target not billable, or $0 base).</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -6602,8 +6388,7 @@
         <is>
           <t>1. QuickBooks connected; the Fee item is NOT mapped in Settings → QuickBooks.
 2. The Discount item IS mapped.
-3. An open WO is available.
-(Ref: FD-QB-004 — VIU pending: verify on staging once deployed.)</t>
+3. An open WO is available.</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -6650,8 +6435,7 @@
       <c r="E126" s="2" t="inlineStr">
         <is>
           <t>1. QuickBooks connected; the Discount item is NOT mapped; the Fee item IS mapped.
-2. An open WO is available.
-(Ref: FD-QB-005 — VIU pending: verify on staging once deployed.)</t>
+2. An open WO is available.</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -6697,9 +6481,7 @@
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; Fee item UNMAPPED.
-(Ref: FD-QB-006 — VIU pending: verify on staging once deployed.)
-Note: Some of these surfaces (labor/part/part-sale) are primarily Group A scope; this case covers the guard breadth.</t>
+          <t>1. QuickBooks connected; Fee item UNMAPPED.</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -6743,8 +6525,7 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; Fee item UNMAPPED.
-(Ref: FD-QB-007 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. QuickBooks connected; Fee item UNMAPPED.</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -6790,8 +6571,7 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>1. Scenario A: QuickBooks connected with Fee item unmapped; scenario B: QuickBooks NOT connected.
-(Ref: FD-QB-008 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. Scenario A: QuickBooks connected with Fee item unmapped; scenario B: QuickBooks NOT connected.</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -6837,8 +6617,7 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected with mapped Fee item; a WO with a fee is ready to invoice/sync.
-(Ref: FD-QB-009 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. QuickBooks connected with mapped Fee item; a WO with a fee is ready to invoice/sync.</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
@@ -6886,9 +6665,7 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected with a location Class set; a WO with fees/discounts is invoiced.
-(Ref: FD-QB-010 — VIU pending: verify on staging once deployed.)
-Note: Per-class allocation is out of scope for V1.</t>
+          <t>1. QuickBooks connected with a location Class set; a WO with fees/discounts is invoiced.</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -6933,8 +6710,7 @@
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; the location's Class has been deleted/deactivated in QuickBooks.
-(Ref: FD-QB-011 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. QuickBooks connected; the location's Class has been deleted/deactivated in QuickBooks.</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
@@ -6979,9 +6755,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; a WO has $100.00 taxable parts and $10.00 tax.
-(Ref: FD-QB-012 — VIU pending: verify on staging once deployed.)
-Note: Uses the spec's exact $100/$10/$150 worked example.</t>
+          <t>1. QuickBooks connected; a WO has $100.00 taxable parts and $10.00 tax.</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -7028,8 +6802,7 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; a WO where stacked MULTIPLE discount lines drive the net subtotal below $0.00 (floor applies).
-(Ref: FD-QB-013 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. QuickBooks connected; a WO where stacked MULTIPLE discount lines drive the net subtotal below $0.00 (floor applies).</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -7076,8 +6849,7 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>1. A WO where discounts will exceed the net subtotal.
-(Ref: FD-QB-014 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO where discounts will exceed the net subtotal.</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
@@ -7123,8 +6895,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; a WO where the floor applied (from FD-QB-012, $50.00 excess).
-(Ref: FD-QB-015 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. QuickBooks connected; a WO where the floor applied (from FD-QB-012, $50.00 excess).</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -7171,8 +6942,7 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; a WO has one taxable fee and one non-taxable fee; the WO is invoiced.
-(Ref: FD-QB-016 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. QuickBooks connected; a WO has one taxable fee and one non-taxable fee; the WO is invoiced.</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
@@ -7217,8 +6987,7 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>1. You have View History Logs and can add/edit/remove adjustments on an open WO.
-(Ref: FD-HIST-001 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. You have View History Logs and can add/edit/remove adjustments on an open WO.</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -7266,9 +7035,7 @@
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>1. A WO has (a) a whole-WO 10% fee named "Env Fee", (b) a labor-line $5.00 flat fee, (c) a part-line discount.
-(Ref: FD-HIST-002 — VIU pending: verify on staging once deployed.)
-Note: History log uses "Full invoice" whereas other screens say "Whole Work Order". Amount is the set rate, not resolved — this is why SFD does not gate the log (S10-R6c).</t>
+          <t>1. A WO has (a) a whole-WO 10% fee named "Env Fee", (b) a labor-line $5.00 flat fee, (c) a part-line discount.</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
@@ -7316,8 +7083,7 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>1. A WO has at least one whole-WO adjustment and one line-level adjustment logged.
-(Ref: FD-HIST-003 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO has at least one whole-WO adjustment and one line-level adjustment logged.</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
@@ -7342,7 +7108,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Verify fee/discount history stays visible when the F&amp;D UI is hidden by the feature flag</t>
+          <t>Verify fee/discount history stays visible when the F&amp;D UI is hidden by the Fees &amp; Discounts feature</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -7363,9 +7129,7 @@
       <c r="E141" s="2" t="inlineStr">
         <is>
           <t>1. A WO already has fee/discount history entries.
-2. The Fees &amp; Discounts feature flag is then turned OFF for the org.
-(Ref: FD-HIST-004 — VIU pending: verify on staging once deployed.)
-Note: The history log is the one exception to the flag-off rule.</t>
+2. The Fees &amp; Discounts feature is then turned OFF for the org.</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -7412,9 +7176,7 @@
       <c r="E142" s="2" t="inlineStr">
         <is>
           <t>1. A WO has fee/discount history entries.
-2. A ZZAUTOTEST role is assigned to Tech with View History Logs ON but See Financial Data OFF (exact-user-match).
-(Ref: FD-HIST-005 — VIU pending: verify on staging once deployed.)
-Note: CAUTION: Story 13 model may not be live on staging yet. Restore Tech to Time Clock (role 77b069d1-...) after.</t>
+2. A ZZAUTOTEST role is assigned to Tech with View History Logs ON but See Financial Data OFF (exact-user-match).</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
@@ -7462,9 +7224,7 @@
       <c r="E143" s="2" t="inlineStr">
         <is>
           <t>1. A WO has fee/discount history.
-2. A ZZAUTOTEST role is assigned to Tech WITHOUT View History Logs (exact-user-match).
-(Ref: FD-HIST-006 — VIU pending: verify on staging once deployed.)
-Note: Restore Tech to Time Clock after. CAUTION: Story 13 model may not be fully live on staging — record actual gating.</t>
+2. A ZZAUTOTEST role is assigned to Tech WITHOUT View History Logs (exact-user-match).</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
@@ -7509,9 +7269,7 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>1. A WO carries a Processing Fee (via auto-apply or customer default).
-(Ref: FD-HIST-007 — VIU pending: verify on staging once deployed.)
-Note: CURRENT-BUILD DIFFERENCE (§14 item 6): current build may show raw "processing_fee" on "Applied to:" instead of "Full invoice" — record actual value.</t>
+          <t>1. A WO carries a Processing Fee (via auto-apply or customer default).</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
@@ -7558,8 +7316,7 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>1. A WO has a whole-WO 10% fee.
-(Ref: FD-HIST-008 — VIU pending: verify on staging once deployed.)</t>
+          <t>1. A WO has a whole-WO 10% fee.</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
@@ -7605,9 +7362,7 @@
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in with a role that has See Financial Data and Work Orders: Create and Edit.
-2. An open work order (not Invoiced/Paid, not in history mode) exists whose relevant base equals exactly $150.00 (e.g. net labor total = $150.00). Mark any throwaway data ZZAUTOTEST.
-(Ref: FD-CALC-001 — VIU pending: verify on staging once deployed.)
-Note: Design open question: the mock Add modal has NO calculation-base selector and computes % against a single flat WO total (design §9.1). Spec §5-R4 requires the base to depend on scope/method. Verify staging actually offers % of Labor Total / Parts Total / Subtotal and resolves against the correct base.</t>
+2. An open work order (not Invoiced/Paid, not in history mode) exists whose relevant base equals exactly $150.00 (e.g. net labor total = $150.00). Mark any throwaway data ZZAUTOTEST.</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
@@ -7659,9 +7414,7 @@
       <c r="E147" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and Work Orders: Create and Edit.
-2. An open work order whose target base equals exactly $33.33.
-(Ref: FD-CALC-002 — VIU pending: verify on staging once deployed.)
-Note: Rounding is a §5 enforced rule not modeled in the design mock. Confirm the server, not just the preview, rounds half-cent up.</t>
+2. An open work order whose target base equals exactly $33.33.</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
@@ -7713,9 +7466,7 @@
       <c r="E148" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data plus the matching change permission.
-2. An open work order with at least one labor line.
-(Ref: FD-CALC-003 — VIU pending: verify on staging once deployed.)
-Note: Open question (requirements §14 item 2): §5-R4's base table lists explicit bases only for the three percentage methods; Whole-WO Flat Amount base = "the set amount" by inference. Confirm no explicit Whole-WO Flat base row is expected.</t>
+2. An open work order with at least one labor line.</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
@@ -7764,9 +7515,7 @@
       <c r="E149" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and Work Order Lines: Create and Edit.
-2. An open work order with a part whose quantity = 3.
-(Ref: FD-CALC-004 — VIU pending: verify on staging once deployed.)
-Note: Part Line Flat is the only Flat method that multiplies by quantity (§5-R14). Whole-WO and Labor Line Flat do not.</t>
+2. An open work order with a part whose quantity = 3.</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
@@ -7816,9 +7565,7 @@
       <c r="E150" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order.
-(Ref: FD-CALC-005 — VIU pending: verify on staging once deployed.)
-Note: Design mock shows no inline error copy for over-100% discounts (design §10). Capture the actual error message/behavior on staging.</t>
+2. An open work order.</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
@@ -7869,9 +7616,7 @@
       <c r="E151" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order.
-(Ref: FD-CALC-006 — VIU pending: verify on staging once deployed.)
-Note: Design's Add button stays disabled when Amount is 0 (design §6), which enforces "&gt; 0" but does not distinguish the $0.01 / 0.01% floor. Verify the exact floor on staging.</t>
+2. An open work order.</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
@@ -7920,9 +7665,7 @@
       <c r="E152" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order whose target base = $100.00.
-(Ref: FD-CALC-007 — VIU pending: verify on staging once deployed.)
-Note: Design difference: the mock labels the field "Max cap" (spec label is "Max Amount (Optional)") and shows it unconditionally, even capping Flat amounts (design §9 item 4). Spec restricts Max Amount to percentage methods only. Verify staging hides it for Flat Amount.</t>
+2. An open work order whose target base = $100.00.</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
@@ -7974,9 +7717,7 @@
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
 2. An open work order whose target base = $100.00.
-3. Note: a $0 Max Amount can normally only come from old data — an entered 0 is treated as empty in the current dialogs (S2-R25).
-(Ref: FD-CALC-008 — VIU pending: verify on staging once deployed.)
-Note: Two behaviors of "0" that must not be confused: typed 0 = empty/no cap (S2-R25); a stored 0 from legacy data forces $0 (§5-R6). Min Amount exists in the data model only, always sent null by both dialogs.</t>
+3. Note: a $0 Max Amount can normally only come from old data — an entered 0 is treated as empty in the current dialogs (S2-R25).</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
@@ -8025,9 +7766,7 @@
       <c r="E154" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order with a target line whose base is $0.00 (e.g. a declined/not-billable labor line, §5-R12).
-(Ref: FD-CALC-009 — VIU pending: verify on staging once deployed.)
-Note: QuickBooks sync (Story 6) is backend and not in the design mocks. Verify the skip at invoice/export time.</t>
+2. An open work order with a target line whose base is $0.00 (e.g. a declined/not-billable labor line, §5-R12).</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
@@ -8076,9 +7815,7 @@
       <c r="E155" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order where an earlier discount has already driven a net total to or below $0 for a whole-WO percentage base.
-(Ref: FD-CALC-010 — VIU pending: verify on staging once deployed.)
-Note: The design preview floors negative amounts to 0 (design §6), consistent with §5. This case is about the BASE being floored, not the whole-total floor (that is FD-CALC-016/017).</t>
+2. An open work order where an earlier discount has already driven a net total to or below $0 for a whole-WO percentage base.</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
@@ -8126,9 +7863,7 @@
       <c r="E156" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order for a taxable customer with a known tax rate and a taxable base.
-(Ref: FD-CALC-011 — VIU pending: verify on staging once deployed.)
-Note: Design open question: the mock Add/Edit dialog collects NO Taxable field (design §9 item 2); spec §1/S2-R26 require a Taxable Yes/No dropdown (default Yes). Verify staging has a Taxable control in the dialog. Preview footer should read "Tax is recalculated on save." (S2-R35).</t>
+2. An open work order for a taxable customer with a known tax rate and a taxable base.</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
@@ -8178,9 +7913,7 @@
       <c r="E157" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data plus both change permissions.
-2. An open work order with gross labor = $200.00 and gross parts = $100.00 (spec worked example).
-(Ref: FD-CALC-012 — VIU pending: verify on staging once deployed.)
-Note: Design mock's preview is base-blind (design §9 item 1). This case validates the enforced §5-R5 step order on the server, not the preview.</t>
+2. An open work order with gross labor = $200.00 and gross parts = $100.00 (spec worked example).</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -8231,9 +7964,7 @@
         <is>
           <t>1. Role has Settings → Finance to create the template and See Financial Data to view amounts.
 2. A Processing Fee template exists: Type = Processing Fee, Calculation type = % of Grand Total, Percent = 3%, marked auto-apply or set as a customer default (a Processing Fee cannot be added to a WO by hand, S8-R16).
-3. An open work order whose net subtotal after line discounts = $300.00 with pre-fee tax = $24.00 (Grand Total base = $324.00).
-(Ref: FD-CALC-013 — VIU pending: verify on staging once deployed.)
-Note: Design does not mock Processing Fee at all (design §9 item 3); it is template/admin-only. On a WO a Processing Fee is remove-only, no Edit (S8-R17); current build reportedly still shows a failing Edit control (requirements §14 item 6).</t>
+3. An open work order whose net subtotal after line discounts = $300.00 with pre-fee tax = $24.00 (Grand Total base = $324.00).</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -8282,9 +8013,7 @@
       <c r="E159" s="2" t="inlineStr">
         <is>
           <t>1. Role has Settings → Finance and See Financial Data.
-2. On the template admin page, open the Processing Fee template create/edit dialog.
-(Ref: FD-CALC-014 — VIU pending: verify on staging once deployed.)
-Note: % of Grand Total is offered only for a Processing Fee (S8-R9). With multiple Processing Fees, each uses the same base excluding every Processing Fee's amount and tax (§5-R4).</t>
+2. On the template admin page, open the Processing Fee template create/edit dialog.</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -8336,9 +8065,7 @@
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
 2. An open work order with $100.00 taxable parts and $10.00 tax (spec worked example).
-3. Location has an active QuickBooks connection (to verify the credit memo).
-(Ref: FD-CALC-015 — VIU pending: verify on staging once deployed.)
-Note: Over-discounting flow is backend/QuickBooks (Story 6) and not in the design mocks. Capture the exact warning text and confirm the credit memo is marked tax-exempt.</t>
+3. Location has an active QuickBooks connection (to verify the credit memo).</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
@@ -8390,9 +8117,7 @@
       <c r="E161" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order with $100.00 taxable parts and $10.00 tax (same base as FD-CALC-015).
-(Ref: FD-CALC-016 — VIU pending: verify on staging once deployed.)
-Note: Reaching a $0.00 total with no tax requires the discount to be taxable and large enough to zero the taxable amount (S6-R10c).</t>
+2. An open work order with $100.00 taxable parts and $10.00 tax (same base as FD-CALC-015).</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
@@ -8443,9 +8168,7 @@
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
 2. Location has an active QuickBooks connection.
-3. An open work order with a small net subtotal and two or more discount lines whose combined size exceeds it.
-(Ref: FD-CALC-017 — VIU pending: verify on staging once deployed.)
-Note: Largest-remainder penny allocation is a backend QuickBooks-sync detail (S6-R10d). Verify line sums equal the floored subtotal to the cent.</t>
+3. An open work order with a small net subtotal and two or more discount lines whose combined size exceeds it.</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
@@ -8495,9 +8218,7 @@
       <c r="E163" s="2" t="inlineStr">
         <is>
           <t>1. A work order (and a part sale, and a customer) already has adjustments to view.
-2. Two ZZAUTOTEST custom roles ready: Role A WITH See Financial Data; Role B WITHOUT See Financial Data (otherwise identical). Use exact-user-match when assigning to Tech (Tech /change staff_id 6fb22c1b-…).
-(Ref: FD-PERM-001 — VIU pending: verify on staging once deployed.)
-Note: Standing rule: restore Tech to Time Clock after permission testing. History-log entries are NOT gated by SFD (they show the set rate, not a resolved total) — see FD-PERM-009.</t>
+2. Two ZZAUTOTEST custom roles ready: Role A WITH See Financial Data; Role B WITHOUT See Financial Data (otherwise identical). Use exact-user-match when assigning to Tech (Tech /change staff_id 6fb22c1b-…).</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
@@ -8547,9 +8268,7 @@
       <c r="E164" s="2" t="inlineStr">
         <is>
           <t>1. An open work order.
-2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Orders: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-002 — VIU pending: verify on staging once deployed.)
-Note: Current-build difference (requirements §10.4): the app may use one WO-edit check where S13-R3/R4 split whole-WO from line-level. Record which permission staging actually enforces.</t>
+2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Orders: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -8598,9 +8317,7 @@
       <c r="E165" s="2" t="inlineStr">
         <is>
           <t>1. An open work order with a labor line and a part.
-2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Order Lines: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-003 — VIU pending: verify on staging once deployed.)
-Note: See current-build split caveat in FD-PERM-002 notes (requirements §10.4).</t>
+2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Work Order Lines: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -8649,9 +8366,7 @@
       <c r="E166" s="2" t="inlineStr">
         <is>
           <t>1. An open part sale with at least one part.
-2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Part Sales: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-004 — VIU pending: verify on staging once deployed.)
-Note: Part Sale does not use Labor Line scope (S11-R2b); a labor-based method resolves to $0 (S11-R2a).</t>
+2. Two ZZAUTOTEST roles, both with See Financial Data ON: Role A WITH Part Sales: Create and Edit; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -8700,9 +8415,7 @@
       <c r="E167" s="2" t="inlineStr">
         <is>
           <t>1. An open work order.
-2. A ZZAUTOTEST role that HAS Work Orders: Create and Edit (and/or Work Order Lines / Part Sales Create and Edit) but has See Financial Data OFF. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-005 — VIU pending: verify on staging once deployed.)
-Note: SFD is a prerequisite for ALL adjustment actions because the controls sit on money-visibility screens. Confirm the server also rejects a crafted request without SFD.</t>
+2. A ZZAUTOTEST role that HAS Work Orders: Create and Edit (and/or Work Order Lines / Part Sales Create and Edit) but has See Financial Data OFF. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
@@ -8751,9 +8464,7 @@
       <c r="E168" s="2" t="inlineStr">
         <is>
           <t>1. An open work order with an existing whole-WO adjustment.
-2. A ZZAUTOTEST role with See Financial Data ON and Work Orders: Create and Edit ON, but with the Work Orders "Delete" permission OFF. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-006 — VIU pending: verify on staging once deployed.)
-Note: Design wording is inconsistent (design §9 item 7): the customer tab and parts breakdown say "Remove", but the inline line/part ⋮ and WO card say "Delete"/"Edit". Regardless of the word shown, the governing permission is Create and Edit. Capture the actual label per surface.</t>
+2. A ZZAUTOTEST role with See Financial Data ON and Work Orders: Create and Edit ON, but with the Work Orders "Delete" permission OFF. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
@@ -8801,9 +8512,7 @@
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>1. Two ZZAUTOTEST roles: Role A WITH Settings → Finance; Role B WITHOUT it. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-007 — VIU pending: verify on staging once deployed.)
-Note: Current-build difference (requirements §10.4 / S7-R7b): the admin page is shown today to any user with a location; S13-R8 tightens it to Settings → Finance. Record which staging enforces.</t>
+          <t>1. Two ZZAUTOTEST roles: Role A WITH Settings → Finance; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F169" s="2" t="inlineStr">
@@ -8852,9 +8561,7 @@
       <c r="E170" s="2" t="inlineStr">
         <is>
           <t>1. A customer exists.
-2. Three ZZAUTOTEST roles: (A) both permissions ON; (B) Customer Management ON but Manage AP/AR OFF; (C) Manage AP/AR ON but Customer Management OFF. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-008 — VIU pending: verify on staging once deployed.)
-Note: Project CLAUDE.md note: per Sasha's spec updates, Manage AP/AR no longer gates aging reports — but it IS still the gate (with Customer Management) for customer F&amp;D defaults per S13-R9. Verify staging enforces both.</t>
+2. Three ZZAUTOTEST roles: (A) both permissions ON; (B) Customer Management ON but Manage AP/AR OFF; (C) Manage AP/AR ON but Customer Management OFF. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -8905,15 +8612,13 @@
       <c r="E171" s="2" t="inlineStr">
         <is>
           <t>1. A work order already has fee/discount history (add/edit/remove entries).
-2. Two ZZAUTOTEST roles: Role A WITH View History Logs; Role B WITHOUT it. Assign by exact-user-match to Tech.
-(Ref: FD-PERM-009 — VIU pending: verify on staging once deployed.)
-Note: Current-build difference (requirements §14 item 6): history "Applied to:" reportedly shows raw "processing_fee" instead of "Full invoice" for a Processing Fee. Verify labels on staging.</t>
+2. Two ZZAUTOTEST roles: Role A WITH View History Logs; Role B WITHOUT it. Assign by exact-user-match to Tech.</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
           <t>1. With Role A: open the WO history log and locate the fee/discount entries.
-2. Also confirm entries remain visible even when the F&amp;D UI is hidden (feature flag off, or See Financial Data off).
+2. Also confirm entries remain visible even when the F&amp;D UI is hidden (Fees &amp; Discounts feature off, or See Financial Data off).
 3. With Role B: open the WO history log.
 4. Restore Tech to Time Clock after.</t>
         </is>
@@ -8921,7 +8626,7 @@
       <c r="G171" s="2" t="inlineStr">
         <is>
           <t>1. With View History Logs ON: fee/discount entries are visible in the history log.
-2. Entries stay visible even when the F&amp;D UI is hidden by the feature flag or by See Financial Data (S10-R1).
+2. Entries stay visible even when the F&amp;D UI is hidden by the Fees &amp; Discounts feature or by See Financial Data (S10-R1).
 3. The log shows the SET rate (e.g. "10.00%" or "$5.00"), not a resolved total, so See Financial Data does NOT gate it (S10-R6c).
 4. With View History Logs OFF: the fee/discount history entries are not shown.</t>
         </is>
@@ -8937,7 +8642,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Verify BOTH gates are required — the FeesAndDiscounts flag ON AND the matching permission</t>
+          <t>Verify BOTH gates are required — the Fees &amp; Discounts feature ON AND the matching permission</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -8957,11 +8662,9 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>1. Ability to toggle the FeesAndDiscounts feature flag for the org (Administration → Feature Flags).
+          <t>1. Ability to toggle the Fees &amp; Discounts feature for the org.
 2. A ZZAUTOTEST role with See Financial Data and Work Orders: Create and Edit ON.
-3. An open work order.
-(Ref: FD-PERM-010 — VIU pending: verify on staging once deployed.)
-Note: The two gates are independent: the flag decides the feature exists (per org); the permission decides what a user may do. Fees &amp; Discounts adds no permission of its own (S13-R1).</t>
+3. An open work order.</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
@@ -8977,12 +8680,12 @@
           <t>1. Flag OFF (regardless of permission): NO F&amp;D controls anywhere (except the history log, Story 10).
 2. Flag ON but permission OFF: controls hidden / action rejected.
 3. Flag ON AND permission ON: controls appear and the action succeeds.
-4. A user needs BOTH the per-org feature flag and the permission (S13-R1).</t>
+4. A user needs BOTH the per-org Fees &amp; Discounts feature and the permission (S13-R1).</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>S13-R1, feature flag + permission (both gates)</t>
+          <t>S13-R1, Fees &amp; Discounts feature + permission (both gates)</t>
         </is>
       </c>
       <c r="I172" s="2" t="inlineStr"/>
@@ -9012,9 +8715,7 @@
       <c r="E173" s="2" t="inlineStr">
         <is>
           <t>1. The user has all F&amp;D permissions (so only the WO state should block).
-2. An Invoiced or Paid work order, and separately a way to enter history mode.
-(Ref: FD-PERM-011 — VIU pending: verify on staging once deployed.)
-Note: OPEN QUESTION (requirements §14 item 3): the spec does not define what puts a user in "history mode." Flag this — the history-mode portion of the step cannot be made concrete until the trigger is confirmed on staging.</t>
+2. An Invoiced or Paid work order, and separately a way to enter history mode.</t>
         </is>
       </c>
       <c r="F173" s="2" t="inlineStr">
@@ -9043,7 +8744,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Verify with the FeesAndDiscounts flag OFF, all F&amp;D UI and behavior are hidden everywhere</t>
+          <t>Verify with the Fees &amp; Discounts feature OFF, all F&amp;D UI and behavior are hidden everywhere</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -9063,16 +8764,14 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>1. Ability to set the FeesAndDiscounts feature flag OFF for the org.
+          <t>1. Ability to set the Fees &amp; Discounts feature OFF for the org.
 2. The test user has See Financial Data and all Create and Edit permissions.
-3. Surfaces to inspect: WO (toolbar ⋯, labor-line ⋮, part menu, sidebar card, Stats tab, Financial Info row), Part Sale (F&amp;D column), Customer (F&amp;D tab), Administration → Service (templates).
-(Ref: FD-FLAG-001 — VIU pending: verify on staging once deployed.)
-Note: The one exception is the WO history log (covered by FD-FLAG-002). On the current staging build the flag is ON but the feature is not yet deployed (viu-findings.md) — re-verify deploy state before running.</t>
+3. Surfaces to inspect: WO (toolbar ⋯, labor-line ⋮, part menu, sidebar card, Stats tab, Financial Info row), Part Sale (F&amp;D column), Customer (F&amp;D tab), Administration → Service (templates).</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>1. Set the feature flag OFF for the org.
+          <t>1. Set the Fees &amp; Discounts feature OFF for the org.
 2. Visit every surface above and look for any F&amp;D control, card, column, tab, or amount.
 3. Restore the flag to its original state after.</t>
         </is>
@@ -9086,7 +8785,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>§1 feature flag, S13-R1</t>
+          <t>§1 Fees &amp; Discounts feature, S13-R1</t>
         </is>
       </c>
       <c r="I174" s="2" t="inlineStr"/>
@@ -9095,7 +8794,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Verify the WO history log STILL shows fee/discount entries even when the feature flag is OFF</t>
+          <t>Verify the WO history log STILL shows fee/discount entries even when the Fees &amp; Discounts feature is OFF</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -9117,14 +8816,12 @@
         <is>
           <t>1. A work order already has fee/discount history entries.
 2. The user has View History Logs.
-3. Ability to set the FeesAndDiscounts flag OFF.
-(Ref: FD-FLAG-002 — VIU pending: verify on staging once deployed.)
-Note: History entries show the set rate, not a resolved dollar total, so they are not gated by See Financial Data either (S10-R6c).</t>
+3. Ability to set the Fees &amp; Discounts feature OFF.</t>
         </is>
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>1. Set the feature flag OFF.
+          <t>1. Set the Fees &amp; Discounts feature OFF.
 2. Open the WO history log and look for the previously-recorded fee/discount entries.
 3. Restore the flag after.</t>
         </is>
@@ -9167,9 +8864,7 @@
       <c r="E176" s="2" t="inlineStr">
         <is>
           <t>1. Two ZZAUTOTEST roles: one with the F&amp;D-relevant permissions, one without.
-2. An open work order.
-(Ref: FD-FLAG-003 — VIU pending: verify on staging once deployed.)
-Note: This is the flag-side complement of FD-PERM-010; keep both to document the flag ON + permission-required interaction from each direction.</t>
+2. An open work order.</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
@@ -9188,7 +8883,7 @@
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>§1 feature flag + S13-R1</t>
+          <t>§1 Fees &amp; Discounts feature + S13-R1</t>
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr"/>
@@ -9218,9 +8913,7 @@
       <c r="E177" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order; open the Add Fee / Discount dialog.
-(Ref: FD-VAL-001 — VIU pending: verify on staging once deployed.)
-Note: Design difference: the mock dialog also has NO base selector and NO Taxable control (design §9 items 1–2). Spec adds Taxable (default Yes, S2-R26) and scope-dependent Calculation type options (§5-R10). Verify the real dialog's enable rule against these extra fields.</t>
+2. An open work order; open the Add Fee / Discount dialog.</t>
         </is>
       </c>
       <c r="F177" s="2" t="inlineStr">
@@ -9271,9 +8964,7 @@
       <c r="E178" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. Add dialog open with Name and Type and Calculation type filled.
-(Ref: FD-VAL-002 — VIU pending: verify on staging once deployed.)
-Note: Design mock shows no inline error copy — only the disabled Add button (design §10). Capture the actual inline error text/behavior on staging.</t>
+2. Add dialog open with Name and Type and Calculation type filled.</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
@@ -9322,9 +9013,7 @@
       <c r="E179" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. Add dialog open with Type, Calculation type, and a valid Amount filled.
-(Ref: FD-VAL-003 — VIU pending: verify on staging once deployed.)
-Note: Verify the exact 100-character enforcement (hard cap vs error) on staging.</t>
+2. Add dialog open with Type, Calculation type, and a valid Amount filled.</t>
         </is>
       </c>
       <c r="F179" s="2" t="inlineStr">
@@ -9373,9 +9062,7 @@
       <c r="E180" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. Add dialog open.
-(Ref: FD-VAL-004 — VIU pending: verify on staging once deployed.)
-Note: Same rule as FD-CALC-005 but framed as dialog validation. Capture the exact rejection UX on staging.</t>
+2. Add dialog open.</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -9425,9 +9112,7 @@
       <c r="E181" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. Add dialog open with Name, Type, Calculation type set.
-(Ref: FD-VAL-005 — VIU pending: verify on staging once deployed.)
-Note: Design mock silently floors negatives to 0 in the preview (design §6) and has no negative-input error state (design §10). Confirm the real dialog rejects negatives rather than silently flooring.</t>
+2. Add dialog open with Name, Type, Calculation type set.</t>
         </is>
       </c>
       <c r="F181" s="2" t="inlineStr">
@@ -9474,9 +9159,7 @@
       <c r="E182" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. Add dialog open.
-(Ref: FD-VAL-006 — VIU pending: verify on staging once deployed.)
-Note: Design difference: the mock labels the field "Max cap", shows it for ALL methods, and caps Flat amounts (design §9 item 4). Spec restricts Max Amount to percentage methods only. Verify staging matches the spec (hidden for Flat).</t>
+2. Add dialog open.</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
@@ -9525,9 +9208,7 @@
       <c r="E183" s="2" t="inlineStr">
         <is>
           <t>1. A template at the location is marked auto-apply (S7-R5).
-2. The SAME template is also set as a default for a customer (S9-R2).
-(Ref: FD-VAL-007 — VIU pending: verify on staging once deployed.)
-Note: OPEN QUESTION / KNOWN BUG (requirements §14 item 4, S9 note): treat a double-add as a KNOWN DEFECT, not a spec requirement; log it in the VIU tab rather than marking the case Failed against spec. Related: a user may deliberately apply the same template to one WO more than once by hand (that is allowed, §1).</t>
+2. The SAME template is also set as a default for a customer (S9-R2).</t>
         </is>
       </c>
       <c r="F183" s="2" t="inlineStr">

</xml_diff>

<commit_message>
F&D + Simple Flow imports: strip internal case-ID cross-references from cells
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/fees-discounts-v1-testrail-import.xlsx
+++ b/testrail-import/fees-discounts-v1-testrail-import.xlsx
@@ -634,7 +634,7 @@
 2. Preview row label flips to 'Discount' and shows −$857.23 (8% × 10,715.39 = 857.2312, rounded to nearest cent = 857.23; §5-R3).
 3. Preview row 'New Work Order Total' shows $9,858.16.
 4. The bottom of the preview reads 'Tax is recalculated on save.' (S2-R35).
-5. The discount amount is signed and colored (see FD-WO-015 for the exact color, which differs spec vs design).</t>
+5. The discount amount is signed and colored (the exact color differs between spec and design).</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -2515,7 +2515,7 @@
       <c r="E43" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. An open work order with 5 adjustments as in FD-FIN-001.</t>
+2. An open work order with 5 adjustments of mixed scope.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2899,7 +2899,7 @@
       <c r="E51" s="2" t="inlineStr">
         <is>
           <t>1. Logged in with See Financial Data.
-2. The #55073 breakdown modal from FD-PCOL-004 is open (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).</t>
+2. The #55073 breakdown modal is open (Parts Handling Fee +$1.43, Military Discount −$3.31, Early Payment Discount −$0.99).</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -6895,7 +6895,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>1. QuickBooks connected; a WO where the floor applied (from FD-QB-012, $50.00 excess).</t>
+          <t>1. QuickBooks connected; a WO where the floor applied (with a $50.00 excess carried as credit).</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -8117,7 +8117,7 @@
       <c r="E161" s="2" t="inlineStr">
         <is>
           <t>1. Role has See Financial Data and the matching change permission.
-2. An open work order with $100.00 taxable parts and $10.00 tax (same base as FD-CALC-015).</t>
+2. An open work order with $100.00 taxable parts and $10.00 tax.</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
@@ -8132,7 +8132,7 @@
           <t>1. A taxable $150.00 discount lowers the taxable amount to $0.00.
 2. Tax = $0.00 (S6-R10c).
 3. Customer pays $0.00 total.
-4. Contrast with FD-CALC-015 (non-taxable) where the $10.00 tax is still owed.</t>
+4. By contrast, when the same discount is non-taxable the $10.00 tax is still owed.</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr">
@@ -8429,7 +8429,7 @@
         <is>
           <t>1. Even with the change permission ON, add/edit/remove is NOT reachable while See Financial Data is OFF (S13-R6).
 2. The controls sit on screens that are hidden when SFD is off, so there is no way to add/edit/remove.
-3. Dollar amounts are also hidden (per FD-PERM-001).</t>
+3. Dollar amounts are also hidden.</t>
         </is>
       </c>
       <c r="H167" s="2" t="inlineStr">
@@ -8829,7 +8829,7 @@
       <c r="G175" s="2" t="inlineStr">
         <is>
           <t>1. Fee/discount history entries REMAIN visible in the WO history log even with the flag off (S10-R1) — the documented exception to "flag off hides everything."
-2. All other F&amp;D UI is still hidden (per FD-FLAG-001).</t>
+2. All other F&amp;D UI is still hidden.</t>
         </is>
       </c>
       <c r="H175" s="2" t="inlineStr">
@@ -8878,7 +8878,7 @@
         <is>
           <t>1. Flag ON alone is not sufficient — without the permission, amounts are hidden and controls are unreachable.
 2. Once the permission is granted, the controls appear and the action works.
-3. Confirms the flag and permission are two independent, both-required gates (cross-reference FD-PERM-010).</t>
+3. Confirms the flag and permission are two independent, both-required gates.</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Apply API-folder rule to Fees & Discounts; switch Simple Flow update generator to XML default
- F&D: add api_related boolean to all 182 cases (2 flagged: FD-CUST-017, FD-PROC-010)
- F&D gen_import.py: route api_related cases to "API — <leaf area>" sections
- Regenerated F&D TestRail CSV/XLSX (182 rows, 0 VIU, 0 feature-flag, 2 API sections)
- Simple Flow gen_update.py: default output format now TestRail XML (--format csv still available)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/fees-discounts-v1-testrail-import.xlsx
+++ b/testrail-import/fees-discounts-v1-testrail-import.xlsx
@@ -4235,7 +4235,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Customer Fees &amp; Discounts tab — negative</t>
+          <t>API — Customer Fees &amp; Discounts tab — negative</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -5496,7 +5496,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Processing Fee — negative</t>
+          <t>API — Processing Fee — negative</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">

</xml_diff>

<commit_message>
spec-monitor: add TestRail import (XML + ID-augmented CSV) for both projects; on-change regen wired into runbook
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testrail-import/fees-discounts-v1-testrail-import.xlsx
+++ b/testrail-import/fees-discounts-v1-testrail-import.xlsx
@@ -3594,14 +3594,14 @@
       <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. Open the customer, go to the Fees &amp; Discounts tab, click "Add Fee/Discount".
-2. In the picker titled "Add Fee/Discount" with caption "Select a fee or discount template to add to this customer.", tick the checkbox for "ZZAUTOTEST Fleet Discount".
-3. Click "Add".</t>
+2. In the picker, open the "Fee / Discount Templates" dropdown and select "ZZAUTOTEST Fleet Discount" (templates are added one at a time).
+3. Click "Save".</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>1. The picker lists each available template as a row with a checkbox plus Name, Type, Calculation Type, Amount.
-2. After clicking Add, the picker closes and a success toast reads exactly "Fee / discount added." (fades on its own).
+          <t>1. The picker is a single-select dropdown listing the available templates — one template is picked and added at a time (adding one at a time is the intended behavior).
+2. After clicking Save, the picker closes and a success toast reads exactly "Fee / discount added." (fades on its own).
 3. "ZZAUTOTEST Fleet Discount" now appears as a row in the Default Fees &amp; Discounts table and the tab count increases by 1.
 4. The added default's columns match the template: Type Discount, Calculation Type % of Subtotal, Amount −10%.</t>
         </is>
@@ -3617,7 +3617,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Verify multi-select adding of several templates at once shows the plural toast</t>
+          <t>Verify several templates are added as customer defaults one at a time (no multi-select)</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3644,20 +3644,20 @@
       <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. Open the customer, Fees &amp; Discounts tab, click "Add Fee/Discount".
-2. Tick the checkboxes for 3 templates.
-3. Click "Add".</t>
+2. Select the first template from the dropdown and click "Save".
+3. Repeat the add for the second and third templates, one at a time.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>1. All 3 selected templates are linked in one action.
-2. A success toast reads exactly "3 fees / discounts added." (the [N] is the number selected).
-3. All 3 appear in the Default Fees &amp; Discounts table; the tab count increases by 3.</t>
+          <t>1. The picker allows only ONE template per add — there is no way to tick several at once (adding one at a time is the intended behavior, so a user cannot accidentally add multiples).
+2. Each add closes the picker and shows its own success toast "Fee / discount added."
+3. After the three adds, all 3 templates appear in the Default Fees &amp; Discounts table and the tab count increases by 3.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>S9-R20, S9-R21, S9-R23b</t>
+          <t>S9-R20, S9-R21, S9-R23a</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -3693,14 +3693,15 @@
       <c r="F67" s="2" t="inlineStr">
         <is>
           <t>1. Open the customer, Fees &amp; Discounts tab, click "Add Fee/Discount".
-2. Review the list of templates offered.</t>
+2. Open the "Fee / Discount Templates" dropdown and review the list of templates offered.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>1. The already-linked template (a) does NOT appear in the picker.
-2. The unlinked Fee/Discount template (b) appears.
-3. The Processing Fee template (c) DOES appear (a Processing Fee can be a customer default), and in the current build its Type column shows "Fee".</t>
+          <t>1. The picker is a single-select dropdown — templates are added one at a time (this is the intended behavior).
+2. The already-linked template (a) does NOT appear in the picker.
+3. The unlinked Fee/Discount template (b) appears.
+4. The Processing Fee template (c) DOES appear (a Processing Fee can be a customer default), and in the current build its Type column shows "Fee".</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3745,7 +3746,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>1. The picker shows exactly "No templates available to add." and no selectable rows.</t>
+          <t>1. The picker's template dropdown shows the "No results" empty state and offers no selectable templates to add.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3759,7 +3760,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Verify removing a customer default via the row menu needs no confirm and toasts</t>
+          <t>Verify removing a customer default via the row's remove action needs no confirm and toasts</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3785,13 +3786,13 @@
       <c r="F69" s="2" t="inlineStr">
         <is>
           <t>1. Open the customer, Fees &amp; Discounts tab.
-2. On a default row, open the 3-dot (⋮) actions menu.
-3. Click "Remove".</t>
+2. On a default row, locate the remove (trash) action.
+3. Click the remove (trash) icon.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>1. The row menu offers only one item, "Remove" (no inline Edit, no "Delete").
+          <t>1. Each default row offers a direct remove (trash) action only (no inline Edit, no separate "Delete").
 2. No confirmation dialog appears; the default is removed immediately.
 3. A success toast reads exactly "Fee / discount removed."
 4. The row disappears and the tab count decreases by 1.</t>
@@ -4215,8 +4216,8 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>1. Intended result: exactly ONE "ZZAUTOTEST Env Fee" adjustment on the WO.
-2. Known bug: it may be added TWICE depending on internal order — record actual count.</t>
+          <t>1. Exactly ONE "ZZAUTOTEST Env Fee" adjustment appears on the new work order.
+2. No second copy of the same template's adjustment is added — the single add is the settled intended behavior (a duplicate would be a defect).</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -4640,7 +4641,8 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>1. In addition to the standard message, the dialog adds exactly: "This template is set as a default for 2 customer(s). Deleting it will remove it from them." (N reflects the actual number of customers).</t>
+          <t>1. The standardized "Delete Template" confirmation dialog opens (the same standardized delete confirmation used elsewhere in Settings, e.g. for pricing matrices).
+2. The dialog includes the warning: "This template is set as a default for 2 customer(s). Deleting it will remove it from them." — the number reflects how many customers currently have the template as a default.</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -9187,7 +9189,7 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Verify a template that is BOTH location auto-apply and a customer default yields ONE adjustment on a new WO (known double-add bug)</t>
+          <t>Verify a template that is BOTH location auto-apply and a customer default yields ONE adjustment on a new WO</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -9220,8 +9222,8 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>1. Intended result: the adjustment appears exactly ONCE on the new WO (§14 item 4 / S9 known gap).
-2. Known bug: the current build may add it TWICE depending on internal order — record the actual count.</t>
+          <t>1. The shared template's adjustment appears exactly ONCE on the new work order — the auto-apply and customer-default paths do not stack.
+2. No duplicate copy is added (the single add is the settled intended behavior; a double-add would be a defect).</t>
         </is>
       </c>
       <c r="H183" s="2" t="inlineStr">

</xml_diff>